<commit_message>
Release v1.0.0: Ending sequence, Sakura skills, size balance, and release configuration
</commit_message>
<xml_diff>
--- a/android/app/src/main/assets/public/files/event/event.xlsx
+++ b/android/app/src/main/assets/public/files/event/event.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\.antigravity\game\files\event\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E9D892-94F6-4946-9C78-3459259E8181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A9AD9A1-4F95-4685-82F2-B08F41F209FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="360" windowWidth="26205" windowHeight="14850" firstSheet="6" activeTab="14" xr2:uid="{77204450-B393-4813-8750-11762B8571B3}"/>
+    <workbookView xWindow="675" yWindow="315" windowWidth="26205" windowHeight="14850" firstSheet="6" activeTab="14" xr2:uid="{77204450-B393-4813-8750-11762B8571B3}"/>
   </bookViews>
   <sheets>
     <sheet name="1207event" sheetId="3" r:id="rId1"/>
@@ -28,6 +28,7 @@
     <sheet name="2RDEVIL" sheetId="14" r:id="rId13"/>
     <sheet name="DOJO" sheetId="16" r:id="rId14"/>
     <sheet name="JIKU" sheetId="17" r:id="rId15"/>
+    <sheet name="Sheet2" sheetId="18" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="377">
   <si>
     <t>今日は12月14日。</t>
     <rPh sb="0" eb="2">
@@ -2183,6 +2184,209 @@
     </rPh>
     <rPh sb="27" eb="28">
       <t>ハジ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>天隕晶</t>
+    <rPh sb="0" eb="1">
+      <t>テン</t>
+    </rPh>
+    <rPh sb="1" eb="2">
+      <t>オ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>アキラ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>七星宝剣</t>
+    <rPh sb="0" eb="1">
+      <t>ナナ</t>
+    </rPh>
+    <rPh sb="1" eb="2">
+      <t>ホシ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ホウケン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>弱点属性の敵への攻撃のダメージを2倍にする。</t>
+    <rPh sb="0" eb="2">
+      <t>ジャクテン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ゾクセイ</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>テキ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>コウゲキ</t>
+    </rPh>
+    <rPh sb="17" eb="18">
+      <t>バイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>攻撃力+5 CH率+5 CH倍率+5</t>
+    <rPh sb="0" eb="3">
+      <t>コウゲキリョク</t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t>リツ</t>
+    </rPh>
+    <rPh sb="14" eb="16">
+      <t>バイリツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>現在精神力の1/10を攻撃力に加算する</t>
+    <rPh sb="0" eb="2">
+      <t>ゲンザイ</t>
+    </rPh>
+    <rPh sb="2" eb="5">
+      <t>セイシンリョク</t>
+    </rPh>
+    <rPh sb="11" eb="14">
+      <t>コウゲキリョク</t>
+    </rPh>
+    <rPh sb="15" eb="17">
+      <t>カサン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>物理攻撃には適用されない。</t>
+    <rPh sb="0" eb="2">
+      <t>ブツリ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>コウゲキ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>テキヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>物理攻撃にのみ適用される。</t>
+    <rPh sb="0" eb="2">
+      <t>ブツリ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>コウゲキ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>テキヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>精神力+5 リロード+5 CH率+5</t>
+    <rPh sb="0" eb="3">
+      <t>セイシンリョク</t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t>リツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>現在生命力の1/10を攻撃力に加算する</t>
+    <rPh sb="0" eb="2">
+      <t>ゲンザイ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>セイメイ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>チカラ</t>
+    </rPh>
+    <rPh sb="11" eb="14">
+      <t>コウゲキリョク</t>
+    </rPh>
+    <rPh sb="15" eb="17">
+      <t>カサン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>生命力+5 回避+5 CH倍率+5</t>
+    <rPh sb="0" eb="3">
+      <t>セイメイリョク</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>カイヒ</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>バイリツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>妙見鑑</t>
+    <rPh sb="0" eb="2">
+      <t>ミョウケン</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>カガミ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>フェイスエリアの奥深くにあるスターストーンを見てからスカイツリーに行くと手に入る。</t>
+    <rPh sb="8" eb="10">
+      <t>オクフカ</t>
+    </rPh>
+    <rPh sb="22" eb="23">
+      <t>ミ</t>
+    </rPh>
+    <rPh sb="33" eb="34">
+      <t>イ</t>
+    </rPh>
+    <rPh sb="36" eb="37">
+      <t>テ</t>
+    </rPh>
+    <rPh sb="38" eb="39">
+      <t>ハイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>スケルトンエリアを下った先にあるキャリバーンを見てから上野にいくと手に入る。</t>
+    <rPh sb="9" eb="10">
+      <t>クダ</t>
+    </rPh>
+    <rPh sb="12" eb="13">
+      <t>サキ</t>
+    </rPh>
+    <rPh sb="23" eb="24">
+      <t>ミ</t>
+    </rPh>
+    <rPh sb="27" eb="29">
+      <t>ウエノ</t>
+    </rPh>
+    <rPh sb="33" eb="34">
+      <t>テ</t>
+    </rPh>
+    <rPh sb="35" eb="36">
+      <t>ハイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>地下21階にある。</t>
+    <rPh sb="0" eb="2">
+      <t>チカ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>カイ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -3480,6 +3684,87 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27536E43-80CF-4D3F-9264-77E06E30D30F}">
+  <dimension ref="A1:A18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
+        <v>372</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{297D6DA5-2661-4E45-AB92-D2EA5AC3D0F2}">
   <dimension ref="A1:A53"/>

</xml_diff>